<commit_message>
Fixes to align load profiles
</commit_message>
<xml_diff>
--- a/InputData/elec/LFHVM/Load Factor Hourly Variance Multiplier.xlsx
+++ b/InputData/elec/LFHVM/Load Factor Hourly Variance Multiplier.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\황일서\Dropbox\NEXT Group\20. 프로젝트 관리\2025 에너지 수요전망 모형 구축\EPS 모형\eps-southkorea-3.3.1\InputData\elec\LFHVM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\South Korea\Models\eps-southkorea\InputData\elec\LFHVM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4BB62AD-7088-4E54-9332-9F1B3AC72369}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08671D1D-3072-47A9-B2B3-0D9301D9F721}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{E755D2B6-154D-4132-AE62-7719D42AA9EA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{E755D2B6-154D-4132-AE62-7719D42AA9EA}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -148,11 +148,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -160,7 +160,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -168,7 +168,7 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -176,13 +176,13 @@
       <i/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -190,7 +190,7 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -242,8 +242,8 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="표준" xfId="0" builtinId="0"/>
-    <cellStyle name="하이퍼링크" xfId="1" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -259,7 +259,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 테마">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -556,17 +556,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86AFABDF-6A59-4ED9-8641-463A0343EC57}">
   <dimension ref="A1:G19"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="43.09765625" customWidth="1"/>
+    <col min="2" max="2" width="43.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -574,7 +574,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7">
       <c r="B4" t="s">
         <v>3</v>
       </c>
@@ -582,7 +582,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7">
       <c r="B5" s="3">
         <v>2021</v>
       </c>
@@ -590,7 +590,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7">
       <c r="B6" t="s">
         <v>5</v>
       </c>
@@ -598,52 +598,52 @@
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7">
       <c r="B7" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:7">
       <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7">
       <c r="A11" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:7">
       <c r="A12" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:7">
       <c r="A13" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:7">
       <c r="A14" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:7">
       <c r="A16" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:1">
       <c r="A17" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:1">
       <c r="A18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:1">
       <c r="A19" t="s">
         <v>13</v>
       </c>
@@ -664,13 +664,13 @@
     <tabColor theme="8" tint="-0.499984740745262"/>
   </sheetPr>
   <dimension ref="A1:I10"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="21.3984375" customWidth="1"/>
-    <col min="2" max="9" width="16.296875" style="6" customWidth="1"/>
+    <col min="1" max="1" width="21.42578125" customWidth="1"/>
+    <col min="2" max="9" width="16.28515625" style="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="34.799999999999997" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:9" ht="30">
       <c r="A1" s="5" t="s">
         <v>27</v>
       </c>
@@ -699,181 +699,181 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
         <v>15</v>
       </c>
       <c r="B2" s="8">
-        <v>0.74</v>
+        <v>0.5</v>
       </c>
       <c r="C2" s="8">
-        <v>0.74</v>
+        <v>0.5</v>
       </c>
       <c r="D2" s="8">
-        <v>0.74</v>
+        <v>0.5</v>
       </c>
       <c r="E2" s="8">
-        <v>0.74</v>
+        <v>0.5</v>
       </c>
       <c r="F2" s="8">
-        <v>0.74</v>
+        <v>0.5</v>
       </c>
       <c r="G2" s="8">
-        <v>0.74</v>
+        <v>0.5</v>
       </c>
       <c r="H2" s="8">
-        <v>0.74</v>
+        <v>0.5</v>
       </c>
       <c r="I2" s="8">
-        <v>0.74</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
       <c r="A3" t="s">
         <v>16</v>
       </c>
       <c r="B3" s="8">
-        <v>0.72</v>
+        <v>0.5</v>
       </c>
       <c r="C3" s="8">
-        <v>0.72</v>
+        <v>0.5</v>
       </c>
       <c r="D3" s="8">
-        <v>0.72</v>
+        <v>0.5</v>
       </c>
       <c r="E3" s="8">
-        <v>0.72</v>
+        <v>0.5</v>
       </c>
       <c r="F3" s="8">
-        <v>0.72</v>
+        <v>0.5</v>
       </c>
       <c r="G3" s="8">
-        <v>0.72</v>
+        <v>0.5</v>
       </c>
       <c r="H3" s="8">
-        <v>0.72</v>
+        <v>0.5</v>
       </c>
       <c r="I3" s="8">
-        <v>0.72</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
       <c r="A4" t="s">
         <v>17</v>
       </c>
       <c r="B4" s="8">
-        <v>0.71</v>
+        <v>0.5</v>
       </c>
       <c r="C4" s="8">
-        <v>0.71</v>
+        <v>0.5</v>
       </c>
       <c r="D4" s="8">
-        <v>0.71</v>
+        <v>0.5</v>
       </c>
       <c r="E4" s="8">
-        <v>0.71</v>
+        <v>0.5</v>
       </c>
       <c r="F4" s="8">
-        <v>0.71</v>
+        <v>0.5</v>
       </c>
       <c r="G4" s="8">
-        <v>0.71</v>
+        <v>0.5</v>
       </c>
       <c r="H4" s="8">
-        <v>0.71</v>
+        <v>0.5</v>
       </c>
       <c r="I4" s="8">
-        <v>0.71</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
       <c r="A5" t="s">
         <v>18</v>
       </c>
       <c r="B5" s="8">
-        <v>0.67</v>
+        <v>0.5</v>
       </c>
       <c r="C5" s="8">
-        <v>0.67</v>
+        <v>0.5</v>
       </c>
       <c r="D5" s="8">
-        <v>0.67</v>
+        <v>0.5</v>
       </c>
       <c r="E5" s="8">
-        <v>0.67</v>
+        <v>0.5</v>
       </c>
       <c r="F5" s="8">
-        <v>0.67</v>
+        <v>0.5</v>
       </c>
       <c r="G5" s="8">
-        <v>0.67</v>
+        <v>0.5</v>
       </c>
       <c r="H5" s="8">
-        <v>0.67</v>
+        <v>0.5</v>
       </c>
       <c r="I5" s="8">
-        <v>0.67</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
       <c r="A6" t="s">
         <v>28</v>
       </c>
       <c r="B6" s="8">
-        <v>0.71</v>
+        <v>0.5</v>
       </c>
       <c r="C6" s="8">
-        <v>0.71</v>
+        <v>0.5</v>
       </c>
       <c r="D6" s="8">
-        <v>0.71</v>
+        <v>0.5</v>
       </c>
       <c r="E6" s="8">
-        <v>0.71</v>
+        <v>0.5</v>
       </c>
       <c r="F6" s="8">
-        <v>0.71</v>
+        <v>0.5</v>
       </c>
       <c r="G6" s="8">
-        <v>0.71</v>
+        <v>0.5</v>
       </c>
       <c r="H6" s="8">
-        <v>0.71</v>
+        <v>0.5</v>
       </c>
       <c r="I6" s="8">
-        <v>0.71</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
       <c r="A7" t="s">
         <v>29</v>
       </c>
       <c r="B7" s="8">
-        <v>0.74</v>
+        <v>0.5</v>
       </c>
       <c r="C7" s="8">
-        <v>0.74</v>
+        <v>0.5</v>
       </c>
       <c r="D7" s="8">
-        <v>0.74</v>
+        <v>0.5</v>
       </c>
       <c r="E7" s="8">
-        <v>0.74</v>
+        <v>0.5</v>
       </c>
       <c r="F7" s="8">
-        <v>0.74</v>
+        <v>0.5</v>
       </c>
       <c r="G7" s="8">
-        <v>0.74</v>
+        <v>0.5</v>
       </c>
       <c r="H7" s="8">
-        <v>0.74</v>
+        <v>0.5</v>
       </c>
       <c r="I7" s="8">
-        <v>0.74</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
       <c r="E10" s="6" t="s">
         <v>30</v>
       </c>
@@ -885,6 +885,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E59C87379D9A4242BB3A95F198D6F941" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="07a235b40ffe2d9a960bde50f6511605">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="40f4d404-d193-41dc-bb72-733c1e774208" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="485fc8e6f691b86ce0aee9b7e82feca0" ns2:_="">
     <xsd:import namespace="40f4d404-d193-41dc-bb72-733c1e774208"/>
@@ -1028,29 +1043,37 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3D209476-3F69-4290-8AA3-E90326FA1916}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69E10275-5E83-4126-B39E-EAA1E3FDA030}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7BEC9438-A445-448D-8D0B-1FB8C589D6E8}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69E10275-5E83-4126-B39E-EAA1E3FDA030}"/>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3D209476-3F69-4290-8AA3-E90326FA1916}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7BEC9438-A445-448D-8D0B-1FB8C589D6E8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="40f4d404-d193-41dc-bb72-733c1e774208"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Calibrated LFHVM using historical data
</commit_message>
<xml_diff>
--- a/InputData/elec/LFHVM/Load Factor Hourly Variance Multiplier.xlsx
+++ b/InputData/elec/LFHVM/Load Factor Hourly Variance Multiplier.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\South Korea\Models\eps-southkorea\InputData\elec\LFHVM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08671D1D-3072-47A9-B2B3-0D9301D9F721}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E38FA707-9466-49EB-9384-8D11BB64B844}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{E755D2B6-154D-4132-AE62-7719D42AA9EA}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{E755D2B6-154D-4132-AE62-7719D42AA9EA}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>LFHVM Load Factor Hourly Variance Multiplier</t>
   </si>
@@ -48,30 +48,9 @@
     <t>Calibrated to peak hour data from:</t>
   </si>
   <si>
-    <t>U.S. Energy Information Administration</t>
-  </si>
-  <si>
-    <t>https://www.eia.gov/todayinenergy/detail.php?id=49216</t>
-  </si>
-  <si>
-    <t>Electricity demand in Lower 48 states reached a high of 720 gigawatthours on August 12</t>
-  </si>
-  <si>
     <t>Notes</t>
   </si>
   <si>
-    <t>NREL's load profiles in SHELF may not reflect the load profiles of real-world experience,</t>
-  </si>
-  <si>
-    <t>even in the United States, and certainly NREL's load profiles will not accurately reflect</t>
-  </si>
-  <si>
-    <t>the load profiles of other countries and regions.  This variable allows hourly variance to</t>
-  </si>
-  <si>
-    <t>be reduce or increased (without altering total load).</t>
-  </si>
-  <si>
     <t>real peak hourly load in the modeled region.  The model must build plants to meet load</t>
   </si>
   <si>
@@ -130,25 +109,26 @@
   </si>
   <si>
     <t>s</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://www.data.go.kr/data/15065266/fileData.do?utm_source=chatgpt.com</t>
-  </si>
-  <si>
-    <t>단순하게 계절별 부하율을 산정</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>부하율 = 평균전력/최대전력</t>
-    <phoneticPr fontId="4" type="noConversion"/>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Korea Power Exchange</t>
+  </si>
+  <si>
+    <t>EPSIS</t>
+  </si>
+  <si>
+    <t>https://epsis.kpx.or.kr/epsisnew/selectEkgeEpsMepChart.do?menuId=030100&amp;locale=eng</t>
+  </si>
+  <si>
+    <t>Peak/Base Demand</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -160,14 +140,6 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -189,7 +161,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -218,31 +189,28 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -555,18 +523,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86AFABDF-6A59-4ED9-8641-463A0343EC57}">
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="43.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -574,87 +542,60 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:2">
       <c r="B4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="B5" s="3">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="B7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="B8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="B5" s="3">
-        <v>2021</v>
-      </c>
-      <c r="G5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="B6" t="s">
-        <v>5</v>
-      </c>
-      <c r="G6" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="B7" s="4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
-      <c r="A10" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
+    </row>
+    <row r="11" spans="1:2">
       <c r="A11" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7">
-      <c r="A16" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1">
-      <c r="A17" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1">
-      <c r="A18" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1">
-      <c r="A19" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
-  <hyperlinks>
-    <hyperlink ref="B7" r:id="rId1" xr:uid="{F03134E3-BA41-4A49-82EE-BA55918987FC}"/>
-  </hyperlinks>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId2"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -667,239 +608,224 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="21.42578125" customWidth="1"/>
-    <col min="2" max="9" width="16.28515625" style="6" customWidth="1"/>
+    <col min="2" max="9" width="16.28515625" style="5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="30">
-      <c r="A1" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B1" s="7" t="s">
+      <c r="A1" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1" s="6" t="s">
         <v>19</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="E1" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F1" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="G1" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="H1" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="I1" s="7" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="C2" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="D2" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="E2" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="F2" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="G2" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="H2" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="I2" s="8">
-        <v>0.5</v>
+        <v>8</v>
+      </c>
+      <c r="B2" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="C2" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="D2" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="E2" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="F2" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="G2" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="H2" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="I2" s="7">
+        <v>0.66</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="C3" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="D3" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="E3" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="F3" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="G3" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="H3" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="I3" s="8">
-        <v>0.5</v>
+        <v>9</v>
+      </c>
+      <c r="B3" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="C3" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="D3" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="E3" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="F3" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="G3" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="H3" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="I3" s="7">
+        <v>0.66</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="C4" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="D4" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="E4" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="F4" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="G4" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="H4" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="I4" s="8">
-        <v>0.5</v>
+        <v>10</v>
+      </c>
+      <c r="B4" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="C4" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="D4" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="E4" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="F4" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="G4" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="H4" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="I4" s="7">
+        <v>0.66</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="C5" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="D5" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="E5" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="F5" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="G5" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="H5" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="I5" s="8">
-        <v>0.5</v>
+        <v>11</v>
+      </c>
+      <c r="B5" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="C5" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="D5" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="E5" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="F5" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="G5" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="H5" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="I5" s="7">
+        <v>0.66</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B6" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="C6" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="D6" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="E6" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="F6" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="G6" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="H6" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="I6" s="8">
-        <v>0.5</v>
+        <v>21</v>
+      </c>
+      <c r="B6" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="C6" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="D6" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="E6" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="F6" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="G6" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="H6" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="I6" s="7">
+        <v>0.66</v>
       </c>
     </row>
     <row r="7" spans="1:9">
       <c r="A7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B7" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="C7" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="D7" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="E7" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="F7" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="G7" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="H7" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="I7" s="8">
-        <v>0.5</v>
+        <v>22</v>
+      </c>
+      <c r="B7" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="C7" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="D7" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="E7" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="F7" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="G7" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="H7" s="7">
+        <v>0.66</v>
+      </c>
+      <c r="I7" s="7">
+        <v>0.66</v>
       </c>
     </row>
     <row r="10" spans="1:9">
-      <c r="E10" s="6" t="s">
-        <v>30</v>
+      <c r="E10" s="5" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E59C87379D9A4242BB3A95F198D6F941" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="07a235b40ffe2d9a960bde50f6511605">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="40f4d404-d193-41dc-bb72-733c1e774208" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="485fc8e6f691b86ce0aee9b7e82feca0" ns2:_="">
     <xsd:import namespace="40f4d404-d193-41dc-bb72-733c1e774208"/>
@@ -1043,24 +969,22 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3D209476-3F69-4290-8AA3-E90326FA1916}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69E10275-5E83-4126-B39E-EAA1E3FDA030}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7BEC9438-A445-448D-8D0B-1FB8C589D6E8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1076,4 +1000,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69E10275-5E83-4126-B39E-EAA1E3FDA030}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3D209476-3F69-4290-8AA3-E90326FA1916}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>